<commit_message>
Laminas regeneradas, informes reconstruidos y baja de laminas_comunales
</commit_message>
<xml_diff>
--- a/output/graficos_dimensiones/comunal_d_dep_a_2018_biobio.xlsx
+++ b/output/graficos_dimensiones/comunal_d_dep_a_2018_biobio.xlsx
@@ -81,7 +81,7 @@
     <t xml:space="preserve">Mulchén</t>
   </si>
   <si>
-    <t xml:space="preserve">Los Alamos</t>
+    <t xml:space="preserve">Los Álamos</t>
   </si>
   <si>
     <t xml:space="preserve">Laja</t>
@@ -111,7 +111,7 @@
     <t xml:space="preserve">Arauco</t>
   </si>
   <si>
-    <t xml:space="preserve">Los Angeles</t>
+    <t xml:space="preserve">Los Ángeles</t>
   </si>
   <si>
     <t xml:space="preserve">Curanilahue</t>
@@ -144,7 +144,7 @@
     <t xml:space="preserve">Fecha de creación</t>
   </si>
   <si>
-    <t xml:space="preserve">2026-10-02 15:30</t>
+    <t xml:space="preserve">2026-10-04 10:27</t>
   </si>
   <si>
     <t xml:space="preserve">Fuente</t>

</xml_diff>

<commit_message>
Laminas regeneradas (regeneracion completa del 2026-10-04), piramides 2018-2024, empates nombrados (#191) (graficos_dimensiones)
</commit_message>
<xml_diff>
--- a/output/graficos_dimensiones/comunal_d_dep_a_2018_biobio.xlsx
+++ b/output/graficos_dimensiones/comunal_d_dep_a_2018_biobio.xlsx
@@ -144,7 +144,7 @@
     <t xml:space="preserve">Fecha de creación</t>
   </si>
   <si>
-    <t xml:space="preserve">2026-10-04 10:27</t>
+    <t xml:space="preserve">2026-10-05 15:43</t>
   </si>
   <si>
     <t xml:space="preserve">Fuente</t>
@@ -937,7 +937,7 @@
         <v>2018</v>
       </c>
       <c r="E23" s="2" t="n">
-        <v>56.62</v>
+        <v>56.63</v>
       </c>
     </row>
     <row r="24">

</xml_diff>